<commit_message>
add strip() at P&ID Tag
</commit_message>
<xml_diff>
--- a/templates/BOM_ULIX_template_rev2.xlsx
+++ b/templates/BOM_ULIX_template_rev2.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ASETS-code\python\pyp-id_finder\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Desktop\pyPidBoMExtractor\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD98A6A9-26E5-4786-9B27-8A4A1A0422C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BCA9466-C315-441D-AB18-7E68B8E27F70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19320" yWindow="-120" windowWidth="19440" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">BOM!$A$1:$V$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">BOM!$A$1:$V$1</definedName>
     <definedName name="A">#REF!</definedName>
     <definedName name="DBWBOM" localSheetId="0">#REF!</definedName>
     <definedName name="DBWBOM">#REF!</definedName>
@@ -111,7 +111,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -129,13 +129,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="7"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -209,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -226,28 +219,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -471,26 +443,26 @@
   <sheetPr>
     <tabColor rgb="FFFFFF99"/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:T6"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.6640625" customWidth="1"/>
-    <col min="2" max="2" width="7.6640625" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" customWidth="1"/>
-    <col min="5" max="5" width="28.33203125" customWidth="1"/>
-    <col min="6" max="6" width="7.88671875" customWidth="1"/>
-    <col min="7" max="7" width="5.6640625" customWidth="1"/>
-    <col min="8" max="8" width="12.5546875" customWidth="1"/>
-    <col min="9" max="10" width="10.21875" customWidth="1"/>
-    <col min="11" max="11" width="11.5546875" customWidth="1"/>
-    <col min="12" max="12" width="12.33203125" customWidth="1"/>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="2" max="2" width="7.7109375" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="28.28515625" customWidth="1"/>
+    <col min="6" max="6" width="7.85546875" customWidth="1"/>
+    <col min="7" max="7" width="5.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" customWidth="1"/>
+    <col min="9" max="10" width="10.28515625" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" customWidth="1"/>
+    <col min="12" max="12" width="12.28515625" customWidth="1"/>
     <col min="13" max="13" width="22" customWidth="1"/>
-    <col min="14" max="14" width="31.88671875" customWidth="1"/>
-    <col min="15" max="20" width="9.109375" customWidth="1"/>
+    <col min="14" max="14" width="31.85546875" customWidth="1"/>
+    <col min="15" max="20" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="19.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -552,55 +524,11 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="7"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="7"/>
-      <c r="S2" s="7"/>
-      <c r="T2" s="6"/>
-    </row>
-    <row r="3" spans="1:20" s="13" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
-      <c r="Q3" s="11"/>
-      <c r="R3" s="11"/>
-      <c r="S3" s="11"/>
-      <c r="T3" s="9"/>
-    </row>
-    <row r="8" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K8" s="13"/>
+    <row r="6" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K6" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:V1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.78740157480314965" bottom="0.78740157480314965" header="0" footer="0"/>

</xml_diff>